<commit_message>
CASE_XPIN XS4 apply: DAILY vol_spot_usd + CASE venue map
- DAILY col vol_spot_usd: 181 rows điền (Feb06-Aug05, GeckoTerminal PancakeSwapV3 0.01%)
- DAILY 147 rows pre-Feb06: ABSTAIN (không có coverage)
- CASE: venue_spot, venue_alpha, spot_perp_ratio, O4_bitmart_vol, detection_floor_spot, verdict_spot_layer

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_XPIN.xlsx
+++ b/docs/case_files/CASE_XPIN.xlsx
@@ -822,7 +822,7 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -869,7 +869,7 @@
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -963,7 +963,7 @@
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -1057,7 +1057,7 @@
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1104,7 @@
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1245,7 @@
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -1292,7 +1292,7 @@
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1339,7 @@
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -1386,7 +1386,7 @@
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -1433,7 +1433,7 @@
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1480,7 @@
       </c>
       <c r="AA17" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -1527,7 +1527,7 @@
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="AA19" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1621,7 @@
       </c>
       <c r="AA20" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -1668,7 +1668,7 @@
       </c>
       <c r="AA21" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -1809,7 +1809,7 @@
       </c>
       <c r="AA24" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -1950,7 +1950,7 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -1997,7 +1997,7 @@
       </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -2044,7 +2044,7 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2091,7 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -2138,7 +2138,7 @@
       </c>
       <c r="AA31" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -2185,7 +2185,7 @@
       </c>
       <c r="AA32" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -2232,7 +2232,7 @@
       </c>
       <c r="AA33" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -2279,7 +2279,7 @@
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -2373,7 +2373,7 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -2420,7 +2420,7 @@
       </c>
       <c r="AA37" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="AA38" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -2514,7 +2514,7 @@
       </c>
       <c r="AA39" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="AA40" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="AA41" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -2655,7 +2655,7 @@
       </c>
       <c r="AA42" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -2702,7 +2702,7 @@
       </c>
       <c r="AA43" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -2749,7 +2749,7 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -2796,7 +2796,7 @@
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -2843,7 +2843,7 @@
       </c>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="AA47" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="AA48" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -2984,7 +2984,7 @@
       </c>
       <c r="AA49" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -3031,7 +3031,7 @@
       </c>
       <c r="AA50" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -3078,7 +3078,7 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -3125,7 +3125,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -3172,7 +3172,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -3219,7 +3219,7 @@
       </c>
       <c r="AA54" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -3266,7 +3266,7 @@
       </c>
       <c r="AA55" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA56" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -3360,7 +3360,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="AA58" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -3454,7 +3454,7 @@
       </c>
       <c r="AA59" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="AA60" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -3548,7 +3548,7 @@
       </c>
       <c r="AA61" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -3595,7 +3595,7 @@
       </c>
       <c r="AA62" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -3642,7 +3642,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -3689,7 +3689,7 @@
       </c>
       <c r="AA64" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -3736,7 +3736,7 @@
       </c>
       <c r="AA65" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -3783,7 +3783,7 @@
       </c>
       <c r="AA66" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -3830,7 +3830,7 @@
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -3877,7 +3877,7 @@
       </c>
       <c r="AA68" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -3924,7 +3924,7 @@
       </c>
       <c r="AA69" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -3971,7 +3971,7 @@
       </c>
       <c r="AA70" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -4018,7 +4018,7 @@
       </c>
       <c r="AA71" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -4065,7 +4065,7 @@
       </c>
       <c r="AA72" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -4112,7 +4112,7 @@
       </c>
       <c r="AA73" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -4159,7 +4159,7 @@
       </c>
       <c r="AA74" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -4206,7 +4206,7 @@
       </c>
       <c r="AA75" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -4253,7 +4253,7 @@
       </c>
       <c r="AA76" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -4300,7 +4300,7 @@
       </c>
       <c r="AA77" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -4347,7 +4347,7 @@
       </c>
       <c r="AA78" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -4394,7 +4394,7 @@
       </c>
       <c r="AA79" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -4441,7 +4441,7 @@
       </c>
       <c r="AA80" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -4488,7 +4488,7 @@
       </c>
       <c r="AA81" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -4535,7 +4535,7 @@
       </c>
       <c r="AA82" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -4582,7 +4582,7 @@
       </c>
       <c r="AA83" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="AA84" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -4676,7 +4676,7 @@
       </c>
       <c r="AA85" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -4723,7 +4723,7 @@
       </c>
       <c r="AA86" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -4770,7 +4770,7 @@
       </c>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -4817,7 +4817,7 @@
       </c>
       <c r="AA88" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -4864,7 +4864,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -4958,7 +4958,7 @@
       </c>
       <c r="AA91" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -5005,7 +5005,7 @@
       </c>
       <c r="AA92" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -5052,7 +5052,7 @@
       </c>
       <c r="AA93" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -5099,7 +5099,7 @@
       </c>
       <c r="AA94" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -5146,7 +5146,7 @@
       </c>
       <c r="AA95" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -5193,7 +5193,7 @@
       </c>
       <c r="AA96" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -5240,7 +5240,7 @@
       </c>
       <c r="AA97" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -5287,7 +5287,7 @@
       </c>
       <c r="AA98" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -5334,7 +5334,7 @@
       </c>
       <c r="AA99" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -5381,7 +5381,7 @@
       </c>
       <c r="AA100" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -5428,7 +5428,7 @@
       </c>
       <c r="AA101" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -5475,7 +5475,7 @@
       </c>
       <c r="AA102" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -5522,7 +5522,7 @@
       </c>
       <c r="AA103" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -5569,7 +5569,7 @@
       </c>
       <c r="AA104" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="AA105" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -5663,7 +5663,7 @@
       </c>
       <c r="AA106" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -5710,7 +5710,7 @@
       </c>
       <c r="AA107" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -5757,7 +5757,7 @@
       </c>
       <c r="AA108" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -5804,7 +5804,7 @@
       </c>
       <c r="AA109" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -5851,7 +5851,7 @@
       </c>
       <c r="AA110" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -5898,7 +5898,7 @@
       </c>
       <c r="AA111" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -5945,7 +5945,7 @@
       </c>
       <c r="AA112" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -5992,7 +5992,7 @@
       </c>
       <c r="AA113" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -6039,7 +6039,7 @@
       </c>
       <c r="AA114" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -6086,7 +6086,7 @@
       </c>
       <c r="AA115" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -6133,7 +6133,7 @@
       </c>
       <c r="AA116" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -6180,7 +6180,7 @@
       </c>
       <c r="AA117" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -6227,7 +6227,7 @@
       </c>
       <c r="AA118" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -6274,7 +6274,7 @@
       </c>
       <c r="AA119" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -6321,7 +6321,7 @@
       </c>
       <c r="AA120" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -6368,7 +6368,7 @@
       </c>
       <c r="AA121" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -6415,7 +6415,7 @@
       </c>
       <c r="AA122" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -6462,7 +6462,7 @@
       </c>
       <c r="AA123" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -6509,7 +6509,7 @@
       </c>
       <c r="AA124" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AA125" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="AA126" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="AA127" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -6697,7 +6697,7 @@
       </c>
       <c r="AA128" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -6744,7 +6744,7 @@
       </c>
       <c r="AA129" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -6791,7 +6791,7 @@
       </c>
       <c r="AA130" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -6838,7 +6838,7 @@
       </c>
       <c r="AA131" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -6885,7 +6885,7 @@
       </c>
       <c r="AA132" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -6932,7 +6932,7 @@
       </c>
       <c r="AA133" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -6979,7 +6979,7 @@
       </c>
       <c r="AA134" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -7026,7 +7026,7 @@
       </c>
       <c r="AA135" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -7073,7 +7073,7 @@
       </c>
       <c r="AA136" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -7120,7 +7120,7 @@
       </c>
       <c r="AA137" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -7167,7 +7167,7 @@
       </c>
       <c r="AA138" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -7214,7 +7214,7 @@
       </c>
       <c r="AA139" t="inlineStr">
         <is>
-          <t>BSC_DEX_only</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -7261,7 +7261,7 @@
       </c>
       <c r="AA140" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -7308,7 +7308,7 @@
       </c>
       <c r="AA141" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="AA142" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -7402,7 +7402,7 @@
       </c>
       <c r="AA143" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -7449,7 +7449,7 @@
       </c>
       <c r="AA144" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -7496,7 +7496,7 @@
       </c>
       <c r="AA145" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -7543,7 +7543,7 @@
       </c>
       <c r="AA146" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -7590,7 +7590,7 @@
       </c>
       <c r="AA147" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -7637,7 +7637,7 @@
       </c>
       <c r="AA148" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -7684,7 +7684,7 @@
       </c>
       <c r="AA149" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
+          <t>BSC_DEX_only_ABSTAIN_pre-Feb06</t>
         </is>
       </c>
     </row>
@@ -7731,8 +7731,11 @@
       </c>
       <c r="AA150" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB150" t="n">
+        <v>1030000</v>
       </c>
     </row>
     <row r="151">
@@ -7778,8 +7781,11 @@
       </c>
       <c r="AA151" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB151" t="n">
+        <v>920000</v>
       </c>
     </row>
     <row r="152">
@@ -7825,8 +7831,11 @@
       </c>
       <c r="AA152" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB152" t="n">
+        <v>345400</v>
       </c>
     </row>
     <row r="153">
@@ -7872,8 +7881,11 @@
       </c>
       <c r="AA153" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB153" t="n">
+        <v>438300</v>
       </c>
     </row>
     <row r="154">
@@ -7919,8 +7931,11 @@
       </c>
       <c r="AA154" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB154" t="n">
+        <v>862400</v>
       </c>
     </row>
     <row r="155">
@@ -7966,8 +7981,11 @@
       </c>
       <c r="AA155" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB155" t="n">
+        <v>749800</v>
       </c>
     </row>
     <row r="156">
@@ -8013,8 +8031,11 @@
       </c>
       <c r="AA156" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB156" t="n">
+        <v>523100</v>
       </c>
     </row>
     <row r="157">
@@ -8060,8 +8081,11 @@
       </c>
       <c r="AA157" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB157" t="n">
+        <v>2510000</v>
       </c>
     </row>
     <row r="158">
@@ -8107,8 +8131,11 @@
       </c>
       <c r="AA158" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB158" t="n">
+        <v>1720000</v>
       </c>
     </row>
     <row r="159">
@@ -8154,8 +8181,11 @@
       </c>
       <c r="AA159" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB159" t="n">
+        <v>1600000</v>
       </c>
     </row>
     <row r="160">
@@ -8201,8 +8231,11 @@
       </c>
       <c r="AA160" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB160" t="n">
+        <v>2290000</v>
       </c>
     </row>
     <row r="161">
@@ -8248,8 +8281,11 @@
       </c>
       <c r="AA161" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB161" t="n">
+        <v>624900</v>
       </c>
     </row>
     <row r="162">
@@ -8295,8 +8331,11 @@
       </c>
       <c r="AA162" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB162" t="n">
+        <v>642900</v>
       </c>
     </row>
     <row r="163">
@@ -8342,8 +8381,11 @@
       </c>
       <c r="AA163" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB163" t="n">
+        <v>1650000</v>
       </c>
     </row>
     <row r="164">
@@ -8389,8 +8431,11 @@
       </c>
       <c r="AA164" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB164" t="n">
+        <v>1240000</v>
       </c>
     </row>
     <row r="165">
@@ -8436,8 +8481,11 @@
       </c>
       <c r="AA165" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB165" t="n">
+        <v>894100</v>
       </c>
     </row>
     <row r="166">
@@ -8483,8 +8531,11 @@
       </c>
       <c r="AA166" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB166" t="n">
+        <v>523700</v>
       </c>
     </row>
     <row r="167">
@@ -8530,8 +8581,11 @@
       </c>
       <c r="AA167" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB167" t="n">
+        <v>1020000</v>
       </c>
     </row>
     <row r="168">
@@ -8577,8 +8631,11 @@
       </c>
       <c r="AA168" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB168" t="n">
+        <v>1210000</v>
       </c>
     </row>
     <row r="169">
@@ -8624,8 +8681,11 @@
       </c>
       <c r="AA169" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB169" t="n">
+        <v>633200</v>
       </c>
     </row>
     <row r="170">
@@ -8671,8 +8731,11 @@
       </c>
       <c r="AA170" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB170" t="n">
+        <v>447700</v>
       </c>
     </row>
     <row r="171">
@@ -8718,8 +8781,11 @@
       </c>
       <c r="AA171" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB171" t="n">
+        <v>450700</v>
       </c>
     </row>
     <row r="172">
@@ -8765,8 +8831,11 @@
       </c>
       <c r="AA172" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB172" t="n">
+        <v>498100</v>
       </c>
     </row>
     <row r="173">
@@ -8812,8 +8881,11 @@
       </c>
       <c r="AA173" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB173" t="n">
+        <v>490300</v>
       </c>
     </row>
     <row r="174">
@@ -8859,8 +8931,11 @@
       </c>
       <c r="AA174" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB174" t="n">
+        <v>546900</v>
       </c>
     </row>
     <row r="175">
@@ -8906,8 +8981,11 @@
       </c>
       <c r="AA175" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB175" t="n">
+        <v>560800</v>
       </c>
     </row>
     <row r="176">
@@ -8953,8 +9031,11 @@
       </c>
       <c r="AA176" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB176" t="n">
+        <v>454200</v>
       </c>
     </row>
     <row r="177">
@@ -8998,8 +9079,11 @@
       </c>
       <c r="AA177" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB177" t="n">
+        <v>421700</v>
       </c>
     </row>
     <row r="178">
@@ -9045,8 +9129,11 @@
       </c>
       <c r="AA178" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB178" t="n">
+        <v>520200</v>
       </c>
     </row>
     <row r="179">
@@ -9092,8 +9179,11 @@
       </c>
       <c r="AA179" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB179" t="n">
+        <v>480300</v>
       </c>
     </row>
     <row r="180">
@@ -9139,8 +9229,11 @@
       </c>
       <c r="AA180" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB180" t="n">
+        <v>436600</v>
       </c>
     </row>
     <row r="181">
@@ -9186,8 +9279,11 @@
       </c>
       <c r="AA181" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB181" t="n">
+        <v>351500</v>
       </c>
     </row>
     <row r="182">
@@ -9233,8 +9329,11 @@
       </c>
       <c r="AA182" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB182" t="n">
+        <v>581800</v>
       </c>
     </row>
     <row r="183">
@@ -9280,8 +9379,11 @@
       </c>
       <c r="AA183" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB183" t="n">
+        <v>718200</v>
       </c>
     </row>
     <row r="184">
@@ -9327,8 +9429,11 @@
       </c>
       <c r="AA184" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB184" t="n">
+        <v>1140000</v>
       </c>
     </row>
     <row r="185">
@@ -9374,8 +9479,11 @@
       </c>
       <c r="AA185" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB185" t="n">
+        <v>3000000</v>
       </c>
     </row>
     <row r="186">
@@ -9421,8 +9529,11 @@
       </c>
       <c r="AA186" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB186" t="n">
+        <v>762300</v>
       </c>
     </row>
     <row r="187">
@@ -9468,8 +9579,11 @@
       </c>
       <c r="AA187" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB187" t="n">
+        <v>387900</v>
       </c>
     </row>
     <row r="188">
@@ -9515,8 +9629,11 @@
       </c>
       <c r="AA188" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB188" t="n">
+        <v>493100</v>
       </c>
     </row>
     <row r="189">
@@ -9562,8 +9679,11 @@
       </c>
       <c r="AA189" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB189" t="n">
+        <v>721500</v>
       </c>
     </row>
     <row r="190">
@@ -9609,8 +9729,11 @@
       </c>
       <c r="AA190" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB190" t="n">
+        <v>669600</v>
       </c>
     </row>
     <row r="191">
@@ -9656,8 +9779,11 @@
       </c>
       <c r="AA191" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB191" t="n">
+        <v>600900</v>
       </c>
     </row>
     <row r="192">
@@ -9703,8 +9829,11 @@
       </c>
       <c r="AA192" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB192" t="n">
+        <v>426000</v>
       </c>
     </row>
     <row r="193">
@@ -9750,8 +9879,11 @@
       </c>
       <c r="AA193" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB193" t="n">
+        <v>458500</v>
       </c>
     </row>
     <row r="194">
@@ -9797,8 +9929,11 @@
       </c>
       <c r="AA194" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB194" t="n">
+        <v>479100</v>
       </c>
     </row>
     <row r="195">
@@ -9844,8 +9979,11 @@
       </c>
       <c r="AA195" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB195" t="n">
+        <v>364600</v>
       </c>
     </row>
     <row r="196">
@@ -9891,8 +10029,11 @@
       </c>
       <c r="AA196" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB196" t="n">
+        <v>253000</v>
       </c>
     </row>
     <row r="197">
@@ -9938,8 +10079,11 @@
       </c>
       <c r="AA197" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB197" t="n">
+        <v>307000</v>
       </c>
     </row>
     <row r="198">
@@ -9985,8 +10129,11 @@
       </c>
       <c r="AA198" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB198" t="n">
+        <v>582800</v>
       </c>
     </row>
     <row r="199">
@@ -10032,8 +10179,11 @@
       </c>
       <c r="AA199" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB199" t="n">
+        <v>523300</v>
       </c>
     </row>
     <row r="200">
@@ -10079,8 +10229,11 @@
       </c>
       <c r="AA200" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB200" t="n">
+        <v>387600</v>
       </c>
     </row>
     <row r="201">
@@ -10126,8 +10279,11 @@
       </c>
       <c r="AA201" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB201" t="n">
+        <v>493700</v>
       </c>
     </row>
     <row r="202">
@@ -10173,8 +10329,11 @@
       </c>
       <c r="AA202" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB202" t="n">
+        <v>261600</v>
       </c>
     </row>
     <row r="203">
@@ -10220,8 +10379,11 @@
       </c>
       <c r="AA203" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB203" t="n">
+        <v>451100</v>
       </c>
     </row>
     <row r="204">
@@ -10267,8 +10429,11 @@
       </c>
       <c r="AA204" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB204" t="n">
+        <v>264100</v>
       </c>
     </row>
     <row r="205">
@@ -10314,8 +10479,11 @@
       </c>
       <c r="AA205" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB205" t="n">
+        <v>380300</v>
       </c>
     </row>
     <row r="206">
@@ -10361,8 +10529,11 @@
       </c>
       <c r="AA206" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB206" t="n">
+        <v>252200</v>
       </c>
     </row>
     <row r="207">
@@ -10408,8 +10579,11 @@
       </c>
       <c r="AA207" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB207" t="n">
+        <v>253400</v>
       </c>
     </row>
     <row r="208">
@@ -10455,8 +10629,11 @@
       </c>
       <c r="AA208" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB208" t="n">
+        <v>213500</v>
       </c>
     </row>
     <row r="209">
@@ -10502,8 +10679,11 @@
       </c>
       <c r="AA209" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB209" t="n">
+        <v>372500</v>
       </c>
     </row>
     <row r="210">
@@ -10549,8 +10729,11 @@
       </c>
       <c r="AA210" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB210" t="n">
+        <v>2260000</v>
       </c>
     </row>
     <row r="211">
@@ -10596,8 +10779,11 @@
       </c>
       <c r="AA211" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB211" t="n">
+        <v>2450000</v>
       </c>
     </row>
     <row r="212">
@@ -10643,8 +10829,11 @@
       </c>
       <c r="AA212" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB212" t="n">
+        <v>3720000</v>
       </c>
     </row>
     <row r="213">
@@ -10690,8 +10879,11 @@
       </c>
       <c r="AA213" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB213" t="n">
+        <v>925400</v>
       </c>
     </row>
     <row r="214">
@@ -10737,8 +10929,11 @@
       </c>
       <c r="AA214" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB214" t="n">
+        <v>618600</v>
       </c>
     </row>
     <row r="215">
@@ -10784,8 +10979,11 @@
       </c>
       <c r="AA215" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB215" t="n">
+        <v>391500</v>
       </c>
     </row>
     <row r="216">
@@ -10831,8 +11029,11 @@
       </c>
       <c r="AA216" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB216" t="n">
+        <v>1620000</v>
       </c>
     </row>
     <row r="217">
@@ -10878,8 +11079,11 @@
       </c>
       <c r="AA217" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB217" t="n">
+        <v>2250000</v>
       </c>
     </row>
     <row r="218">
@@ -10925,8 +11129,11 @@
       </c>
       <c r="AA218" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB218" t="n">
+        <v>1040000</v>
       </c>
     </row>
     <row r="219">
@@ -10972,8 +11179,11 @@
       </c>
       <c r="AA219" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB219" t="n">
+        <v>1110000</v>
       </c>
     </row>
     <row r="220">
@@ -11019,8 +11229,11 @@
       </c>
       <c r="AA220" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB220" t="n">
+        <v>696900</v>
       </c>
     </row>
     <row r="221">
@@ -11066,8 +11279,11 @@
       </c>
       <c r="AA221" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB221" t="n">
+        <v>683800</v>
       </c>
     </row>
     <row r="222">
@@ -11113,8 +11329,11 @@
       </c>
       <c r="AA222" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB222" t="n">
+        <v>517600</v>
       </c>
     </row>
     <row r="223">
@@ -11160,8 +11379,11 @@
       </c>
       <c r="AA223" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB223" t="n">
+        <v>531300</v>
       </c>
     </row>
     <row r="224">
@@ -11207,8 +11429,11 @@
       </c>
       <c r="AA224" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB224" t="n">
+        <v>739400</v>
       </c>
     </row>
     <row r="225">
@@ -11254,8 +11479,11 @@
       </c>
       <c r="AA225" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB225" t="n">
+        <v>1650000</v>
       </c>
     </row>
     <row r="226">
@@ -11301,8 +11529,11 @@
       </c>
       <c r="AA226" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB226" t="n">
+        <v>1060000</v>
       </c>
     </row>
     <row r="227">
@@ -11348,8 +11579,11 @@
       </c>
       <c r="AA227" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB227" t="n">
+        <v>636100</v>
       </c>
     </row>
     <row r="228">
@@ -11395,8 +11629,11 @@
       </c>
       <c r="AA228" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB228" t="n">
+        <v>367200</v>
       </c>
     </row>
     <row r="229">
@@ -11442,8 +11679,11 @@
       </c>
       <c r="AA229" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB229" t="n">
+        <v>514400</v>
       </c>
     </row>
     <row r="230">
@@ -11489,8 +11729,11 @@
       </c>
       <c r="AA230" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB230" t="n">
+        <v>858600</v>
       </c>
     </row>
     <row r="231">
@@ -11536,8 +11779,11 @@
       </c>
       <c r="AA231" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB231" t="n">
+        <v>668200</v>
       </c>
     </row>
     <row r="232">
@@ -11583,8 +11829,11 @@
       </c>
       <c r="AA232" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB232" t="n">
+        <v>569600</v>
       </c>
     </row>
     <row r="233">
@@ -11630,8 +11879,11 @@
       </c>
       <c r="AA233" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB233" t="n">
+        <v>1440000</v>
       </c>
     </row>
     <row r="234">
@@ -11677,8 +11929,11 @@
       </c>
       <c r="AA234" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB234" t="n">
+        <v>392800</v>
       </c>
     </row>
     <row r="235">
@@ -11724,8 +11979,11 @@
       </c>
       <c r="AA235" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB235" t="n">
+        <v>1650000</v>
       </c>
     </row>
     <row r="236">
@@ -11785,8 +12043,11 @@
       </c>
       <c r="AA236" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB236" t="n">
+        <v>919300</v>
       </c>
     </row>
     <row r="237">
@@ -11846,8 +12107,11 @@
       </c>
       <c r="AA237" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB237" t="n">
+        <v>470100</v>
       </c>
     </row>
     <row r="238">
@@ -11907,8 +12171,11 @@
       </c>
       <c r="AA238" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB238" t="n">
+        <v>324100</v>
       </c>
     </row>
     <row r="239">
@@ -11968,8 +12235,11 @@
       </c>
       <c r="AA239" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB239" t="n">
+        <v>648300</v>
       </c>
     </row>
     <row r="240">
@@ -12029,8 +12299,11 @@
       </c>
       <c r="AA240" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB240" t="n">
+        <v>489900</v>
       </c>
     </row>
     <row r="241">
@@ -12090,8 +12363,11 @@
       </c>
       <c r="AA241" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB241" t="n">
+        <v>1230000</v>
       </c>
     </row>
     <row r="242">
@@ -12151,8 +12427,11 @@
       </c>
       <c r="AA242" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB242" t="n">
+        <v>1310000</v>
       </c>
     </row>
     <row r="243">
@@ -12212,8 +12491,11 @@
       </c>
       <c r="AA243" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB243" t="n">
+        <v>1400000</v>
       </c>
     </row>
     <row r="244">
@@ -12273,8 +12555,11 @@
       </c>
       <c r="AA244" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB244" t="n">
+        <v>650200</v>
       </c>
     </row>
     <row r="245">
@@ -12334,8 +12619,11 @@
       </c>
       <c r="AA245" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB245" t="n">
+        <v>1550000</v>
       </c>
     </row>
     <row r="246">
@@ -12395,8 +12683,11 @@
       </c>
       <c r="AA246" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB246" t="n">
+        <v>1420000</v>
       </c>
     </row>
     <row r="247">
@@ -12456,8 +12747,11 @@
       </c>
       <c r="AA247" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB247" t="n">
+        <v>1400000</v>
       </c>
     </row>
     <row r="248">
@@ -12517,8 +12811,11 @@
       </c>
       <c r="AA248" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB248" t="n">
+        <v>2220000</v>
       </c>
     </row>
     <row r="249">
@@ -12578,8 +12875,11 @@
       </c>
       <c r="AA249" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB249" t="n">
+        <v>697100</v>
       </c>
     </row>
     <row r="250">
@@ -12639,8 +12939,11 @@
       </c>
       <c r="AA250" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB250" t="n">
+        <v>809000</v>
       </c>
     </row>
     <row r="251">
@@ -12700,8 +13003,11 @@
       </c>
       <c r="AA251" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB251" t="n">
+        <v>649700</v>
       </c>
     </row>
     <row r="252">
@@ -12761,8 +13067,11 @@
       </c>
       <c r="AA252" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB252" t="n">
+        <v>371400</v>
       </c>
     </row>
     <row r="253">
@@ -12822,8 +13131,11 @@
       </c>
       <c r="AA253" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB253" t="n">
+        <v>308500</v>
       </c>
     </row>
     <row r="254">
@@ -12883,8 +13195,11 @@
       </c>
       <c r="AA254" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB254" t="n">
+        <v>322200</v>
       </c>
     </row>
     <row r="255">
@@ -12944,8 +13259,11 @@
       </c>
       <c r="AA255" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB255" t="n">
+        <v>704300</v>
       </c>
     </row>
     <row r="256">
@@ -13003,8 +13321,11 @@
       </c>
       <c r="AA256" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB256" t="n">
+        <v>390600</v>
       </c>
     </row>
     <row r="257">
@@ -13064,8 +13385,11 @@
       </c>
       <c r="AA257" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB257" t="n">
+        <v>375600</v>
       </c>
     </row>
     <row r="258">
@@ -13125,8 +13449,11 @@
       </c>
       <c r="AA258" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB258" t="n">
+        <v>400700</v>
       </c>
     </row>
     <row r="259">
@@ -13186,8 +13513,11 @@
       </c>
       <c r="AA259" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB259" t="n">
+        <v>634900</v>
       </c>
     </row>
     <row r="260">
@@ -13247,8 +13577,11 @@
       </c>
       <c r="AA260" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB260" t="n">
+        <v>641700</v>
       </c>
     </row>
     <row r="261">
@@ -13308,8 +13641,11 @@
       </c>
       <c r="AA261" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB261" t="n">
+        <v>589800</v>
       </c>
     </row>
     <row r="262">
@@ -13369,8 +13705,11 @@
       </c>
       <c r="AA262" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB262" t="n">
+        <v>859300</v>
       </c>
     </row>
     <row r="263">
@@ -13430,8 +13769,11 @@
       </c>
       <c r="AA263" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB263" t="n">
+        <v>286500</v>
       </c>
     </row>
     <row r="264">
@@ -13491,8 +13833,11 @@
       </c>
       <c r="AA264" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB264" t="n">
+        <v>277800</v>
       </c>
     </row>
     <row r="265">
@@ -13552,8 +13897,11 @@
       </c>
       <c r="AA265" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB265" t="n">
+        <v>496700</v>
       </c>
     </row>
     <row r="266">
@@ -13613,8 +13961,11 @@
       </c>
       <c r="AA266" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB266" t="n">
+        <v>832500</v>
       </c>
     </row>
     <row r="267">
@@ -13674,8 +14025,11 @@
       </c>
       <c r="AA267" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB267" t="n">
+        <v>711100</v>
       </c>
     </row>
     <row r="268">
@@ -13735,8 +14089,11 @@
       </c>
       <c r="AA268" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB268" t="n">
+        <v>882200</v>
       </c>
     </row>
     <row r="269">
@@ -13796,8 +14153,11 @@
       </c>
       <c r="AA269" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB269" t="n">
+        <v>1320000</v>
       </c>
     </row>
     <row r="270">
@@ -13857,8 +14217,11 @@
       </c>
       <c r="AA270" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB270" t="n">
+        <v>1150000</v>
       </c>
     </row>
     <row r="271">
@@ -13918,8 +14281,11 @@
       </c>
       <c r="AA271" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB271" t="n">
+        <v>407200</v>
       </c>
     </row>
     <row r="272">
@@ -13979,8 +14345,11 @@
       </c>
       <c r="AA272" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB272" t="n">
+        <v>580400</v>
       </c>
     </row>
     <row r="273">
@@ -14040,8 +14409,11 @@
       </c>
       <c r="AA273" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB273" t="n">
+        <v>455000</v>
       </c>
     </row>
     <row r="274">
@@ -14101,8 +14473,11 @@
       </c>
       <c r="AA274" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB274" t="n">
+        <v>596500</v>
       </c>
     </row>
     <row r="275">
@@ -14162,8 +14537,11 @@
       </c>
       <c r="AA275" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB275" t="n">
+        <v>597000</v>
       </c>
     </row>
     <row r="276">
@@ -14223,8 +14601,11 @@
       </c>
       <c r="AA276" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB276" t="n">
+        <v>610000</v>
       </c>
     </row>
     <row r="277">
@@ -14284,8 +14665,11 @@
       </c>
       <c r="AA277" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB277" t="n">
+        <v>998300</v>
       </c>
     </row>
     <row r="278">
@@ -14345,8 +14729,11 @@
       </c>
       <c r="AA278" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB278" t="n">
+        <v>451400</v>
       </c>
     </row>
     <row r="279">
@@ -14406,8 +14793,11 @@
       </c>
       <c r="AA279" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB279" t="n">
+        <v>1020000</v>
       </c>
     </row>
     <row r="280">
@@ -14467,8 +14857,11 @@
       </c>
       <c r="AA280" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB280" t="n">
+        <v>715200</v>
       </c>
     </row>
     <row r="281">
@@ -14528,8 +14921,11 @@
       </c>
       <c r="AA281" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB281" t="n">
+        <v>944300</v>
       </c>
     </row>
     <row r="282">
@@ -14589,8 +14985,11 @@
       </c>
       <c r="AA282" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB282" t="n">
+        <v>1130000</v>
       </c>
     </row>
     <row r="283">
@@ -14650,8 +15049,11 @@
       </c>
       <c r="AA283" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB283" t="n">
+        <v>1460000</v>
       </c>
     </row>
     <row r="284">
@@ -14711,8 +15113,11 @@
       </c>
       <c r="AA284" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB284" t="n">
+        <v>551900</v>
       </c>
     </row>
     <row r="285">
@@ -14770,8 +15175,11 @@
       </c>
       <c r="AA285" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB285" t="n">
+        <v>350500</v>
       </c>
     </row>
     <row r="286">
@@ -14831,8 +15239,11 @@
       </c>
       <c r="AA286" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB286" t="n">
+        <v>871100</v>
       </c>
     </row>
     <row r="287">
@@ -14892,8 +15303,11 @@
       </c>
       <c r="AA287" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB287" t="n">
+        <v>1370000</v>
       </c>
     </row>
     <row r="288">
@@ -14953,8 +15367,11 @@
       </c>
       <c r="AA288" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB288" t="n">
+        <v>1140000</v>
       </c>
     </row>
     <row r="289">
@@ -15014,8 +15431,11 @@
       </c>
       <c r="AA289" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB289" t="n">
+        <v>997300</v>
       </c>
     </row>
     <row r="290">
@@ -15085,8 +15505,11 @@
       </c>
       <c r="AA290" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB290" t="n">
+        <v>1010000</v>
       </c>
     </row>
     <row r="291">
@@ -15158,8 +15581,11 @@
       </c>
       <c r="AA291" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB291" t="n">
+        <v>556500</v>
       </c>
     </row>
     <row r="292">
@@ -15233,8 +15659,11 @@
       </c>
       <c r="AA292" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB292" t="n">
+        <v>360000</v>
       </c>
     </row>
     <row r="293">
@@ -15312,8 +15741,11 @@
       </c>
       <c r="AA293" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB293" t="n">
+        <v>491800</v>
       </c>
     </row>
     <row r="294">
@@ -15391,8 +15823,11 @@
       </c>
       <c r="AA294" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB294" t="n">
+        <v>1250000</v>
       </c>
     </row>
     <row r="295">
@@ -15470,8 +15905,11 @@
       </c>
       <c r="AA295" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB295" t="n">
+        <v>2300000</v>
       </c>
     </row>
     <row r="296">
@@ -15551,8 +15989,11 @@
       </c>
       <c r="AA296" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB296" t="n">
+        <v>1010000</v>
       </c>
     </row>
     <row r="297">
@@ -15632,8 +16073,11 @@
       </c>
       <c r="AA297" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB297" t="n">
+        <v>565400</v>
       </c>
     </row>
     <row r="298">
@@ -15713,8 +16157,11 @@
       </c>
       <c r="AA298" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB298" t="n">
+        <v>547700</v>
       </c>
     </row>
     <row r="299">
@@ -15794,8 +16241,11 @@
       </c>
       <c r="AA299" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB299" t="n">
+        <v>399700</v>
       </c>
     </row>
     <row r="300">
@@ -15875,8 +16325,11 @@
       </c>
       <c r="AA300" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB300" t="n">
+        <v>491400</v>
       </c>
     </row>
     <row r="301">
@@ -15956,8 +16409,11 @@
       </c>
       <c r="AA301" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB301" t="n">
+        <v>972700</v>
       </c>
     </row>
     <row r="302">
@@ -16037,8 +16493,11 @@
       </c>
       <c r="AA302" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB302" t="n">
+        <v>1270000</v>
       </c>
     </row>
     <row r="303">
@@ -16118,8 +16577,11 @@
       </c>
       <c r="AA303" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB303" t="n">
+        <v>496677</v>
       </c>
     </row>
     <row r="304">
@@ -16199,8 +16661,11 @@
       </c>
       <c r="AA304" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB304" t="n">
+        <v>2788481</v>
       </c>
     </row>
     <row r="305">
@@ -16280,8 +16745,11 @@
       </c>
       <c r="AA305" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB305" t="n">
+        <v>7785737</v>
       </c>
     </row>
     <row r="306">
@@ -16361,8 +16829,11 @@
       </c>
       <c r="AA306" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB306" t="n">
+        <v>2907977</v>
       </c>
     </row>
     <row r="307">
@@ -16442,8 +16913,11 @@
       </c>
       <c r="AA307" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB307" t="n">
+        <v>1494383</v>
       </c>
     </row>
     <row r="308">
@@ -16523,8 +16997,11 @@
       </c>
       <c r="AA308" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB308" t="n">
+        <v>1270000</v>
       </c>
     </row>
     <row r="309">
@@ -16604,8 +17081,11 @@
       </c>
       <c r="AA309" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB309" t="n">
+        <v>2580000</v>
       </c>
     </row>
     <row r="310">
@@ -16685,8 +17165,11 @@
       </c>
       <c r="AA310" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB310" t="n">
+        <v>1490000</v>
       </c>
     </row>
     <row r="311">
@@ -16766,8 +17249,11 @@
       </c>
       <c r="AA311" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB311" t="n">
+        <v>635100</v>
       </c>
     </row>
     <row r="312">
@@ -16847,8 +17333,11 @@
       </c>
       <c r="AA312" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB312" t="n">
+        <v>1520000</v>
       </c>
     </row>
     <row r="313">
@@ -16928,8 +17417,11 @@
       </c>
       <c r="AA313" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB313" t="n">
+        <v>660300</v>
       </c>
     </row>
     <row r="314">
@@ -17009,8 +17501,11 @@
       </c>
       <c r="AA314" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB314" t="n">
+        <v>759200</v>
       </c>
     </row>
     <row r="315">
@@ -17090,8 +17585,11 @@
       </c>
       <c r="AA315" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB315" t="n">
+        <v>887800</v>
       </c>
     </row>
     <row r="316">
@@ -17171,8 +17669,11 @@
       </c>
       <c r="AA316" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB316" t="n">
+        <v>619700</v>
       </c>
     </row>
     <row r="317">
@@ -17252,8 +17753,11 @@
       </c>
       <c r="AA317" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB317" t="n">
+        <v>656700</v>
       </c>
     </row>
     <row r="318">
@@ -17333,8 +17837,11 @@
       </c>
       <c r="AA318" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB318" t="n">
+        <v>688000</v>
       </c>
     </row>
     <row r="319">
@@ -17414,8 +17921,11 @@
       </c>
       <c r="AA319" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB319" t="n">
+        <v>451800</v>
       </c>
     </row>
     <row r="320">
@@ -17495,8 +18005,11 @@
       </c>
       <c r="AA320" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB320" t="n">
+        <v>582500</v>
       </c>
     </row>
     <row r="321">
@@ -17576,8 +18089,11 @@
       </c>
       <c r="AA321" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB321" t="n">
+        <v>668500</v>
       </c>
     </row>
     <row r="322">
@@ -17657,8 +18173,11 @@
       </c>
       <c r="AA322" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB322" t="n">
+        <v>761300</v>
       </c>
     </row>
     <row r="323">
@@ -17738,8 +18257,11 @@
       </c>
       <c r="AA323" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB323" t="n">
+        <v>472000</v>
       </c>
     </row>
     <row r="324">
@@ -17819,8 +18341,11 @@
       </c>
       <c r="AA324" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB324" t="n">
+        <v>396700</v>
       </c>
     </row>
     <row r="325">
@@ -17900,8 +18425,11 @@
       </c>
       <c r="AA325" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB325" t="n">
+        <v>639300</v>
       </c>
     </row>
     <row r="326">
@@ -17981,8 +18509,11 @@
       </c>
       <c r="AA326" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB326" t="n">
+        <v>228300</v>
       </c>
     </row>
     <row r="327">
@@ -18062,8 +18593,11 @@
       </c>
       <c r="AA327" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB327" t="n">
+        <v>557100</v>
       </c>
     </row>
     <row r="328">
@@ -18143,8 +18677,11 @@
       </c>
       <c r="AA328" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB328" t="n">
+        <v>620900</v>
       </c>
     </row>
     <row r="329">
@@ -18224,8 +18761,11 @@
       </c>
       <c r="AA329" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
-        </is>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
+        </is>
+      </c>
+      <c r="AB329" t="n">
+        <v>326400</v>
       </c>
     </row>
     <row r="330">
@@ -18305,11 +18845,11 @@
       </c>
       <c r="AA330" t="inlineStr">
         <is>
-          <t>Alpha_ALPHA334+BSC_DEX</t>
+          <t>BSC_DEX_PancakeSwapV3_0.01%</t>
         </is>
       </c>
       <c r="AB330" t="n">
-        <v>290000</v>
+        <v>154800</v>
       </c>
     </row>
   </sheetData>
@@ -18329,7 +18869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -18428,7 +18968,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>NONE (no Binance spot) — BSC DEX PancakeSwap V3 0.01% main pool</t>
+          <t>BSC DEX PancakeSwapV3 0.01% main pool (0x08de…4a4, liq=$944K, v24=$345K). 19 ghost pools (all $0 vol). No Binance spot, no CEX spot trustworthy.</t>
         </is>
       </c>
     </row>
@@ -18440,7 +18980,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Binance Alpha ALPHA_334 (listed ~2026-01-27)</t>
+          <t>ALPHA_334 listed ~2026-01-27. API 400 (klines endpoint not serving XPIN). Local store: 0 files. Alpha vol = ABSTAIN.</t>
         </is>
       </c>
     </row>
@@ -18818,7 +19358,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>BSC DEX only ~$286K/day (negligible vs perp)</t>
+          <t>BSC DEX: $521K/day avg crowd_surge (Jul22-Aug05); $1.9M/day prior (Jul8-21). Crowd surge: DEX contracted 0.28x — crowd buying pure perp leverage, not spot. Source: GeckoTerminal Feb06–Aug05 (181 bars). Pre-Feb06: ABSTAIN (no coverage).</t>
         </is>
       </c>
     </row>
@@ -18938,7 +19478,31 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PENDING verify ($1.1B suspicious — likely wash)</t>
+          <t>CoinGecko: BitMart $1.61M vol/liq=338x SUSPECT. Biconomy $251K vol/liq=661x SUSPECT. KuCoin $72K vol/liq=7.2x CLEAN. Gate $198K. MEXC $142K. Hibt $22K vol/liq=6.9x CLEAN. Source: XS1c CoinGecko tickers+depth 06/08/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>detection_floor_spot</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Daily spot total ~$571K (DEX $521K + Alpha $50K est). 1% total supply (1B tokens @ $0.00155) = $1.55M = 2.7x daily spot → DETECTABLE. 5% circ (2.4B tokens) = $3.73M = 6.5x daily spot → VERY DETECTABLE. Any non-trivial kho selling via BSC DEX would be visible within 1 day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>verdict_spot_layer</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>XS4 verdict (06/08/2026): WATCH-nhạt ĐỨNG. Spot thin ($571K/day) confirms crowd buying pure leverage (perp), not real money into DEX. No DEX sell burst observed (XS3b rate-limited; XS3c DEX vol expanded on Jul11 fail = crowd panic buy into DEX, not distribution). Detection floor LOW: any kho &gt;1% supply selling via DEX would be visible within 1-2 days. Verdict unchanged from cold-start X6. Alpha ABSTAIN pending operator verification.</t>
         </is>
       </c>
     </row>

</xml_diff>